<commit_message>
figure update minor revisions
</commit_message>
<xml_diff>
--- a/4-Analysis/results/gha26_inv2.xlsx
+++ b/4-Analysis/results/gha26_inv2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmp/Documents/local-git/wolf_clusters/4-Analysis/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E3402A17-C0DB-E643-B550-DC54AD3C5174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698FE146-B216-924D-A2C7-D05C0E57340F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43440" yWindow="-18300" windowWidth="24420" windowHeight="11400" xr2:uid="{76585D50-6560-D34A-B236-1EC249E04AC4}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{76585D50-6560-D34A-B236-1EC249E04AC4}"/>
   </bookViews>
   <sheets>
     <sheet name="gha26_inv2" sheetId="1" r:id="rId1"/>
@@ -1202,8 +1202,8 @@
         <v>35.558149229919003</v>
       </c>
       <c r="H2" t="str">
-        <f>_xlfn.CONCAT(ROUND(D2,2)," +/-  ", ROUND(G2,2))</f>
-        <v>-37.43 +/-  35.56</v>
+        <f>_xlfn.CONCAT(ROUND(C2,2)," +/-  ", ROUND(G2,2))</f>
+        <v>-28 +/-  35.56</v>
       </c>
       <c r="I2">
         <v>22</v>
@@ -1221,8 +1221,8 @@
         <v>28.987540988246401</v>
       </c>
       <c r="N2" t="str">
-        <f>_xlfn.CONCAT(ROUND(J2,2)," +/-  ", ROUND(M2,2))</f>
-        <v>31.4 +/-  28.99</v>
+        <f>_xlfn.CONCAT(ROUND(I2,2)," +/-  ", ROUND(M2,2))</f>
+        <v>22 +/-  28.99</v>
       </c>
       <c r="O2">
         <v>92</v>
@@ -1240,8 +1240,8 @@
         <v>120.47175396316401</v>
       </c>
       <c r="T2" t="str">
-        <f>_xlfn.CONCAT(ROUND(P2,2)," +/-  ", ROUND(S2,2))</f>
-        <v>127 +/-  120.47</v>
+        <f>_xlfn.CONCAT(ROUND(O2,2)," +/-  ", ROUND(S2,2))</f>
+        <v>92 +/-  120.47</v>
       </c>
       <c r="U2">
         <v>247</v>
@@ -1259,8 +1259,8 @@
         <v>102.533090646581</v>
       </c>
       <c r="Z2" t="str">
-        <f>_xlfn.CONCAT(ROUND(V2,2)," +/-  ", ROUND(Y2,2))</f>
-        <v>238.77 +/-  102.53</v>
+        <f>_xlfn.CONCAT(ROUND(U2,2)," +/-  ", ROUND(Y2,2))</f>
+        <v>247 +/-  102.53</v>
       </c>
       <c r="AA2">
         <v>3</v>
@@ -1278,8 +1278,8 @@
         <v>3.5305203997402699</v>
       </c>
       <c r="AF2" t="str">
-        <f>_xlfn.CONCAT(ROUND(AB2,2)," +/-  ", ROUND(AE2,2))</f>
-        <v>3.74 +/-  3.53</v>
+        <f>_xlfn.CONCAT(ROUND(AA2,2)," +/-  ", ROUND(AE2,2))</f>
+        <v>3 +/-  3.53</v>
       </c>
       <c r="AG2">
         <v>0.421472937000887</v>
@@ -1297,8 +1297,8 @@
         <v>0.26973869030013897</v>
       </c>
       <c r="AL2" t="str">
-        <f>_xlfn.CONCAT(ROUND(AH2*100,2)," +/-  ", ROUND(AK2*100,2))</f>
-        <v>41.66 +/-  26.97</v>
+        <f>_xlfn.CONCAT(ROUND(AG2*100,2)," +/-  ", ROUND(AK2*100,2))</f>
+        <v>42.15 +/-  26.97</v>
       </c>
       <c r="AM2">
         <v>164</v>
@@ -1334,8 +1334,8 @@
         <v>23.3637100909284</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H12" si="0">_xlfn.CONCAT(ROUND(D3,2)," +/-  ", ROUND(G3,2))</f>
-        <v>-25.28 +/-  23.36</v>
+        <f t="shared" ref="H3:H12" si="0">_xlfn.CONCAT(ROUND(C3,2)," +/-  ", ROUND(G3,2))</f>
+        <v>-21 +/-  23.36</v>
       </c>
       <c r="I3">
         <v>5</v>
@@ -1353,8 +1353,8 @@
         <v>9.5579423493899505</v>
       </c>
       <c r="N3" t="str">
-        <f t="shared" ref="N3:N12" si="1">_xlfn.CONCAT(ROUND(J3,2)," +/-  ", ROUND(M3,2))</f>
-        <v>8.53 +/-  9.56</v>
+        <f t="shared" ref="N3:N12" si="1">_xlfn.CONCAT(ROUND(I3,2)," +/-  ", ROUND(M3,2))</f>
+        <v>5 +/-  9.56</v>
       </c>
       <c r="O3">
         <v>32</v>
@@ -1372,8 +1372,8 @@
         <v>68.375501101962101</v>
       </c>
       <c r="T3" t="str">
-        <f t="shared" ref="T3:T12" si="2">_xlfn.CONCAT(ROUND(P3,2)," +/-  ", ROUND(S3,2))</f>
-        <v>55.39 +/-  68.38</v>
+        <f t="shared" ref="T3:T12" si="2">_xlfn.CONCAT(ROUND(O3,2)," +/-  ", ROUND(S3,2))</f>
+        <v>32 +/-  68.38</v>
       </c>
       <c r="U3">
         <v>145.5</v>
@@ -1391,8 +1391,8 @@
         <v>108.788675346177</v>
       </c>
       <c r="Z3" t="str">
-        <f t="shared" ref="Z3:Z12" si="3">_xlfn.CONCAT(ROUND(V3,2)," +/-  ", ROUND(Y3,2))</f>
-        <v>155.93 +/-  108.79</v>
+        <f t="shared" ref="Z3:Z12" si="3">_xlfn.CONCAT(ROUND(U3,2)," +/-  ", ROUND(Y3,2))</f>
+        <v>145.5 +/-  108.79</v>
       </c>
       <c r="AA3">
         <v>1</v>
@@ -1410,8 +1410,8 @@
         <v>2.23047912454637</v>
       </c>
       <c r="AF3" t="str">
-        <f t="shared" ref="AF3:AF12" si="4">_xlfn.CONCAT(ROUND(AB3,2)," +/-  ", ROUND(AE3,2))</f>
-        <v>1.46 +/-  2.23</v>
+        <f t="shared" ref="AF3:AF12" si="4">_xlfn.CONCAT(ROUND(AA3,2)," +/-  ", ROUND(AE3,2))</f>
+        <v>1 +/-  2.23</v>
       </c>
       <c r="AG3">
         <v>0.45903010033444802</v>
@@ -1429,8 +1429,8 @@
         <v>0.37985661081948802</v>
       </c>
       <c r="AL3" t="str">
-        <f t="shared" ref="AL3:AL12" si="5">_xlfn.CONCAT(ROUND(AH3*100,2)," +/-  ", ROUND(AK3*100,2))</f>
-        <v>41.99 +/-  37.99</v>
+        <f t="shared" ref="AL3:AL12" si="5">_xlfn.CONCAT(ROUND(AG3*100,2)," +/-  ", ROUND(AK3*100,2))</f>
+        <v>45.9 +/-  37.99</v>
       </c>
       <c r="AM3">
         <v>260</v>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H4" t="str">
         <f t="shared" si="0"/>
-        <v>-15.29 +/-  39.52</v>
+        <v>-8 +/-  39.52</v>
       </c>
       <c r="I4">
         <v>6</v>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="N4" t="str">
         <f t="shared" si="1"/>
-        <v>8.93 +/-  9.81</v>
+        <v>6 +/-  9.81</v>
       </c>
       <c r="O4">
         <v>16.5</v>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="T4" t="str">
         <f t="shared" si="2"/>
-        <v>44.9 +/-  67.88</v>
+        <v>16.5 +/-  67.88</v>
       </c>
       <c r="U4">
         <v>140</v>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="Z4" t="str">
         <f t="shared" si="3"/>
-        <v>152.61 +/-  92.77</v>
+        <v>140 +/-  92.77</v>
       </c>
       <c r="AA4">
         <v>0</v>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="AF4" t="str">
         <f t="shared" si="4"/>
-        <v>1.01 +/-  1.85</v>
+        <v>0 +/-  1.85</v>
       </c>
       <c r="AG4">
         <v>0</v>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="AL4" t="str">
         <f t="shared" si="5"/>
-        <v>28.46 +/-  35.79</v>
+        <v>0 +/-  35.79</v>
       </c>
       <c r="AM4">
         <v>212</v>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="H5" t="str">
         <f t="shared" si="0"/>
-        <v>-23.92 +/-  19.98</v>
+        <v>-19 +/-  19.98</v>
       </c>
       <c r="I5">
         <v>7</v>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="N5" t="str">
         <f t="shared" si="1"/>
-        <v>9.54 +/-  11.09</v>
+        <v>7 +/-  11.09</v>
       </c>
       <c r="O5">
         <v>15.976699999999999</v>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="T5" t="str">
         <f t="shared" si="2"/>
-        <v>42.83 +/-  62.85</v>
+        <v>15.98 +/-  62.85</v>
       </c>
       <c r="U5">
         <v>121</v>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="Z5" t="str">
         <f t="shared" si="3"/>
-        <v>139.54 +/-  108.56</v>
+        <v>121 +/-  108.56</v>
       </c>
       <c r="AA5">
         <v>0</v>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="AF5" t="str">
         <f t="shared" si="4"/>
-        <v>1.06 +/-  1.99</v>
+        <v>0 +/-  1.99</v>
       </c>
       <c r="AG5">
         <v>0</v>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="AL5" t="str">
         <f t="shared" si="5"/>
-        <v>26.68 +/-  33.09</v>
+        <v>0 +/-  33.09</v>
       </c>
       <c r="AM5">
         <v>385</v>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="H6" t="str">
         <f t="shared" si="0"/>
-        <v>-25.94 +/-  37.47</v>
+        <v>-20 +/-  37.47</v>
       </c>
       <c r="I6">
         <v>8</v>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="N6" t="str">
         <f t="shared" si="1"/>
-        <v>13.89 +/-  15.19</v>
+        <v>8 +/-  15.19</v>
       </c>
       <c r="O6">
         <v>45</v>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="T6" t="str">
         <f t="shared" si="2"/>
-        <v>81.9 +/-  95.7</v>
+        <v>45 +/-  95.7</v>
       </c>
       <c r="U6">
         <v>198</v>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Z6" t="str">
         <f t="shared" si="3"/>
-        <v>198.95 +/-  117.23</v>
+        <v>198 +/-  117.23</v>
       </c>
       <c r="AA6">
         <v>1</v>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="AF6" t="str">
         <f t="shared" si="4"/>
-        <v>2.47 +/-  3.42</v>
+        <v>1 +/-  3.42</v>
       </c>
       <c r="AG6">
         <v>0.53589743589743599</v>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="AL6" t="str">
         <f t="shared" si="5"/>
-        <v>43.46 +/-  35.58</v>
+        <v>53.59 +/-  35.58</v>
       </c>
       <c r="AM6">
         <v>196</v>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="H7" t="str">
         <f t="shared" si="0"/>
-        <v>-28.16 +/-  25.28</v>
+        <v>-21 +/-  25.28</v>
       </c>
       <c r="I7">
         <v>6</v>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="N7" t="str">
         <f t="shared" si="1"/>
-        <v>8.8 +/-  8.44</v>
+        <v>6 +/-  8.44</v>
       </c>
       <c r="O7">
         <v>18</v>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="T7" t="str">
         <f t="shared" si="2"/>
-        <v>48.34 +/-  66.6</v>
+        <v>18 +/-  66.6</v>
       </c>
       <c r="U7">
         <v>146</v>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="Z7" t="str">
         <f t="shared" si="3"/>
-        <v>156.8 +/-  106.14</v>
+        <v>146 +/-  106.14</v>
       </c>
       <c r="AA7">
         <v>1</v>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="AF7" t="str">
         <f t="shared" si="4"/>
-        <v>1.12 +/-  1.81</v>
+        <v>1 +/-  1.81</v>
       </c>
       <c r="AG7">
         <v>0.14835164835164799</v>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="AL7" t="str">
         <f t="shared" si="5"/>
-        <v>32.27 +/-  35.92</v>
+        <v>14.84 +/-  35.92</v>
       </c>
       <c r="AM7">
         <v>230</v>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="H8" t="str">
         <f t="shared" si="0"/>
-        <v>-28.14 +/-  31.34</v>
+        <v>-16 +/-  31.34</v>
       </c>
       <c r="I8">
         <v>16</v>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="N8" t="str">
         <f t="shared" si="1"/>
-        <v>19.33 +/-  13.18</v>
+        <v>16 +/-  13.18</v>
       </c>
       <c r="O8">
         <v>63.001249999999999</v>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="T8" t="str">
         <f t="shared" si="2"/>
-        <v>75.09 +/-  64.63</v>
+        <v>63 +/-  64.63</v>
       </c>
       <c r="U8">
         <v>232.5</v>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="Z8" t="str">
         <f t="shared" si="3"/>
-        <v>233.66 +/-  100.4</v>
+        <v>232.5 +/-  100.4</v>
       </c>
       <c r="AA8">
         <v>1</v>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="AF8" t="str">
         <f t="shared" si="4"/>
-        <v>1.76 +/-  1.8</v>
+        <v>1 +/-  1.8</v>
       </c>
       <c r="AG8">
         <v>0.36237373737373701</v>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="AL8" t="str">
         <f t="shared" si="5"/>
-        <v>34.51 +/-  29.04</v>
+        <v>36.24 +/-  29.04</v>
       </c>
       <c r="AM8">
         <v>92</v>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
-        <v>-29.15 +/-  34.8</v>
+        <v>-20 +/-  34.8</v>
       </c>
       <c r="I9">
         <v>7</v>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="N9" t="str">
         <f t="shared" si="1"/>
-        <v>9.83 +/-  9.33</v>
+        <v>7 +/-  9.33</v>
       </c>
       <c r="O9">
         <v>22</v>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="T9" t="str">
         <f t="shared" si="2"/>
-        <v>46.09 +/-  54.24</v>
+        <v>22 +/-  54.24</v>
       </c>
       <c r="U9">
         <v>141</v>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="Z9" t="str">
         <f t="shared" si="3"/>
-        <v>148.73 +/-  95.92</v>
+        <v>141 +/-  95.92</v>
       </c>
       <c r="AA9">
         <v>0</v>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="AF9" t="str">
         <f t="shared" si="4"/>
-        <v>1.03 +/-  1.62</v>
+        <v>0 +/-  1.62</v>
       </c>
       <c r="AG9">
         <v>0</v>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="AL9" t="str">
         <f t="shared" si="5"/>
-        <v>31.45 +/-  35.8</v>
+        <v>0 +/-  35.8</v>
       </c>
       <c r="AM9">
         <v>175</v>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
-        <v>-28.44 +/-  30.45</v>
+        <v>-18.5 +/-  30.45</v>
       </c>
       <c r="I10">
         <v>13</v>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="N10" t="str">
         <f t="shared" si="1"/>
-        <v>18.21 +/-  15.69</v>
+        <v>13 +/-  15.69</v>
       </c>
       <c r="O10">
         <v>47</v>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="T10" t="str">
         <f t="shared" si="2"/>
-        <v>76.02 +/-  78.92</v>
+        <v>47 +/-  78.92</v>
       </c>
       <c r="U10">
         <v>210.5</v>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="Z10" t="str">
         <f t="shared" si="3"/>
-        <v>209.44 +/-  121.91</v>
+        <v>210.5 +/-  121.91</v>
       </c>
       <c r="AA10">
         <v>1.5</v>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="AF10" t="str">
         <f t="shared" si="4"/>
-        <v>2.25 +/-  3.05</v>
+        <v>1.5 +/-  3.05</v>
       </c>
       <c r="AG10">
         <v>0.224080267558529</v>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="AL10" t="str">
         <f t="shared" si="5"/>
-        <v>36.15 +/-  31.92</v>
+        <v>22.41 +/-  31.92</v>
       </c>
       <c r="AM10">
         <v>48</v>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
-        <v>-46.1 +/-  47.13</v>
+        <v>-30 +/-  47.13</v>
       </c>
       <c r="I11">
         <v>27</v>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="N11" t="str">
         <f t="shared" si="1"/>
-        <v>54.37 +/-  60.51</v>
+        <v>27 +/-  60.51</v>
       </c>
       <c r="O11">
         <v>182</v>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="T11" t="str">
         <f t="shared" si="2"/>
-        <v>277.12 +/-  288.62</v>
+        <v>182 +/-  288.62</v>
       </c>
       <c r="U11">
         <v>241</v>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="Z11" t="str">
         <f t="shared" si="3"/>
-        <v>232.82 +/-  116.66</v>
+        <v>241 +/-  116.66</v>
       </c>
       <c r="AA11">
         <v>5</v>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="AF11" t="str">
         <f t="shared" si="4"/>
-        <v>8.72 +/-  9.44</v>
+        <v>5 +/-  9.44</v>
       </c>
       <c r="AG11">
         <v>0.52941176470588203</v>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="AL11" t="str">
         <f t="shared" si="5"/>
-        <v>46.97 +/-  27.1</v>
+        <v>52.94 +/-  27.1</v>
       </c>
       <c r="AM11">
         <v>105</v>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
-        <v>-58.73 +/-  51.56</v>
+        <v>-47 +/-  51.56</v>
       </c>
       <c r="I12">
         <v>22.5</v>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="N12" t="str">
         <f t="shared" si="1"/>
-        <v>40 +/-  36.91</v>
+        <v>22.5 +/-  36.91</v>
       </c>
       <c r="O12">
         <v>167.00835000000001</v>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="T12" t="str">
         <f t="shared" si="2"/>
-        <v>217.28 +/-  189.3</v>
+        <v>167.01 +/-  189.3</v>
       </c>
       <c r="U12">
         <v>276</v>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="Z12" t="str">
         <f t="shared" si="3"/>
-        <v>255.2 +/-  116.08</v>
+        <v>276 +/-  116.08</v>
       </c>
       <c r="AA12">
         <v>5</v>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="AF12" t="str">
         <f t="shared" si="4"/>
-        <v>7.1 +/-  6.51</v>
+        <v>5 +/-  6.51</v>
       </c>
       <c r="AG12">
         <v>0.58365943945002696</v>
@@ -2618,7 +2618,7 @@
       </c>
       <c r="AL12" t="str">
         <f t="shared" si="5"/>
-        <v>49.85 +/-  30.17</v>
+        <v>58.37 +/-  30.17</v>
       </c>
       <c r="AM12">
         <v>30</v>

</xml_diff>